<commit_message>
Update data: 28 Juli 2026 pukul 08.16 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Report_Dashboard_Morning.xlsx
+++ b/dashboard/public/Report_Dashboard_Morning.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Monitoring Kecamatan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Leaderboard PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Leaderboard PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Leaderboard Kecamatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring Kecamatan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leaderboard PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leaderboard PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leaderboard Kecamatan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,7 +594,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hari/Tanggal : 27 Juli 2026</t>
+          <t>Hari/Tanggal : 28 Juli 2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -616,32 +616,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 08.18 WITA</t>
+          <t>Pukul        : 08.16 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-42):</t>
+          <t>Target Hari Ini (H-44):</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>70.14%</t>
+          <t>73.48%</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Hijau &gt;= 70.14%</t>
+          <t>Hijau &gt;= 73.48%</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Kuning 35.07% - 70.14%</t>
+          <t>Kuning 36.74% - 73.48%</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Merah &lt; 35.07%</t>
+          <t>Merah &lt; 36.74%</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       <c r="P8" s="9" t="n">
         <v>1054</v>
       </c>
-      <c r="Q8" s="11">
+      <c r="Q8" s="12">
         <f>P8/B8</f>
         <v/>
       </c>
@@ -1844,7 +1844,7 @@
         <f>SUM(P7:P21)</f>
         <v/>
       </c>
-      <c r="Q22" s="11">
+      <c r="Q22" s="12">
         <f>P22/B22</f>
         <v/>
       </c>
@@ -1900,7 +1900,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hari/Tanggal : 27 Juli 2026</t>
+          <t>Hari/Tanggal : 28 Juli 2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1917,17 +1917,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 08.18 WITA</t>
+          <t>Pukul        : 08.16 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-42):</t>
+          <t>Target Hari Ini (H-44):</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>70.14%</t>
+          <t>73.48%</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4157,7 @@
       <c r="L52" s="9" t="n">
         <v>343</v>
       </c>
-      <c r="M52" s="11" t="n">
+      <c r="M52" s="12" t="n">
         <v>0.7313432835820897</v>
       </c>
     </row>
@@ -4204,7 +4204,7 @@
       <c r="L53" s="9" t="n">
         <v>369</v>
       </c>
-      <c r="M53" s="11" t="n">
+      <c r="M53" s="12" t="n">
         <v>0.7306930693069308</v>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       <c r="L54" s="9" t="n">
         <v>320</v>
       </c>
-      <c r="M54" s="11" t="n">
+      <c r="M54" s="12" t="n">
         <v>0.7305936073059359</v>
       </c>
     </row>
@@ -4298,7 +4298,7 @@
       <c r="L55" s="9" t="n">
         <v>337</v>
       </c>
-      <c r="M55" s="11" t="n">
+      <c r="M55" s="12" t="n">
         <v>0.7278617710583153</v>
       </c>
     </row>
@@ -4345,7 +4345,7 @@
       <c r="L56" s="9" t="n">
         <v>293</v>
       </c>
-      <c r="M56" s="11" t="n">
+      <c r="M56" s="12" t="n">
         <v>0.7252475247524752</v>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       <c r="L57" s="9" t="n">
         <v>312</v>
       </c>
-      <c r="M57" s="11" t="n">
+      <c r="M57" s="12" t="n">
         <v>0.7188940092165899</v>
       </c>
     </row>
@@ -4439,7 +4439,7 @@
       <c r="L58" s="9" t="n">
         <v>329</v>
       </c>
-      <c r="M58" s="11" t="n">
+      <c r="M58" s="12" t="n">
         <v>0.7167755991285403</v>
       </c>
     </row>
@@ -4486,7 +4486,7 @@
       <c r="L59" s="9" t="n">
         <v>302</v>
       </c>
-      <c r="M59" s="11" t="n">
+      <c r="M59" s="12" t="n">
         <v>0.7156398104265402</v>
       </c>
     </row>
@@ -4533,7 +4533,7 @@
       <c r="L60" s="9" t="n">
         <v>312</v>
       </c>
-      <c r="M60" s="11" t="n">
+      <c r="M60" s="12" t="n">
         <v>0.7155963302752294</v>
       </c>
     </row>
@@ -4580,7 +4580,7 @@
       <c r="L61" s="9" t="n">
         <v>274</v>
       </c>
-      <c r="M61" s="11" t="n">
+      <c r="M61" s="12" t="n">
         <v>0.7154046997389034</v>
       </c>
     </row>
@@ -4627,7 +4627,7 @@
       <c r="L62" s="9" t="n">
         <v>310</v>
       </c>
-      <c r="M62" s="11" t="n">
+      <c r="M62" s="12" t="n">
         <v>0.7126436781609197</v>
       </c>
     </row>
@@ -4674,7 +4674,7 @@
       <c r="L63" s="9" t="n">
         <v>363</v>
       </c>
-      <c r="M63" s="11" t="n">
+      <c r="M63" s="12" t="n">
         <v>0.7103718199608611</v>
       </c>
     </row>
@@ -4721,7 +4721,7 @@
       <c r="L64" s="9" t="n">
         <v>378</v>
       </c>
-      <c r="M64" s="11" t="n">
+      <c r="M64" s="12" t="n">
         <v>0.7091932457786116</v>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       <c r="L65" s="9" t="n">
         <v>321</v>
       </c>
-      <c r="M65" s="11" t="n">
+      <c r="M65" s="12" t="n">
         <v>0.7070484581497797</v>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       <c r="L66" s="9" t="n">
         <v>357</v>
       </c>
-      <c r="M66" s="11" t="n">
+      <c r="M66" s="12" t="n">
         <v>0.7055335968379447</v>
       </c>
     </row>
@@ -4862,7 +4862,7 @@
       <c r="L67" s="9" t="n">
         <v>230</v>
       </c>
-      <c r="M67" s="11" t="n">
+      <c r="M67" s="12" t="n">
         <v>0.7055214723926381</v>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
       <c r="L68" s="9" t="n">
         <v>347</v>
       </c>
-      <c r="M68" s="11" t="n">
+      <c r="M68" s="12" t="n">
         <v>0.7052845528455285</v>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       <c r="L69" s="9" t="n">
         <v>375</v>
       </c>
-      <c r="M69" s="11" t="n">
+      <c r="M69" s="12" t="n">
         <v>0.7048872180451127</v>
       </c>
     </row>
@@ -8149,7 +8149,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hari/Tanggal : 27 Juli 2026</t>
+          <t>Hari/Tanggal : 28 Juli 2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -8166,17 +8166,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 08.18 WITA</t>
+          <t>Pukul        : 08.16 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-42):</t>
+          <t>Target Hari Ini (H-44):</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>70.14%</t>
+          <t>73.48%</t>
         </is>
       </c>
     </row>
@@ -8620,7 +8620,7 @@
       <c r="L14" s="9" t="n">
         <v>2169</v>
       </c>
-      <c r="M14" s="11" t="n">
+      <c r="M14" s="12" t="n">
         <v>0.7298115746971736</v>
       </c>
     </row>
@@ -8667,7 +8667,7 @@
       <c r="L15" s="9" t="n">
         <v>1049</v>
       </c>
-      <c r="M15" s="11" t="n">
+      <c r="M15" s="12" t="n">
         <v>0.7068733153638814</v>
       </c>
     </row>
@@ -8714,7 +8714,7 @@
       <c r="L16" s="9" t="n">
         <v>1760</v>
       </c>
-      <c r="M16" s="11" t="n">
+      <c r="M16" s="12" t="n">
         <v>0.7059767348576013</v>
       </c>
     </row>
@@ -9360,7 +9360,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hari/Tanggal : 27 Juli 2026</t>
+          <t>Hari/Tanggal : 28 Juli 2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -9377,17 +9377,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 08.18 WITA</t>
+          <t>Pukul        : 08.16 WITA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-42):</t>
+          <t>Target Hari Ini (H-44):</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>70.14%</t>
+          <t>73.48%</t>
         </is>
       </c>
     </row>
@@ -9513,7 +9513,7 @@
           <t>Tatoareng</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="12" t="n">
         <v>0.7102425876010782</v>
       </c>
       <c r="D12" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Update data: 3 Agustus 2026 pukul 09.35 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Report_Dashboard_Morning.xlsx
+++ b/dashboard/public/Report_Dashboard_Morning.xlsx
@@ -618,7 +618,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 12.40 WITA</t>
+          <t>Pukul        : 09.35 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1919,7 +1919,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 12.40 WITA</t>
+          <t>Pukul        : 09.35 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -8168,7 +8168,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 12.40 WITA</t>
+          <t>Pukul        : 09.35 WITA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9379,7 +9379,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pukul        : 12.40 WITA</t>
+          <t>Pukul        : 09.35 WITA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update data: 6 Agustus 2026 pukul 08.35 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Report_Dashboard_Morning.xlsx
+++ b/dashboard/public/Report_Dashboard_Morning.xlsx
@@ -623,27 +623,27 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-52):</t>
+          <t>Target Hari Ini (H-53):</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>86.84%</t>
+          <t>88.51%</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Hijau &gt;= 86.84%</t>
+          <t>Hijau &gt;= 88.51%</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Kuning 43.42% - 86.84%</t>
+          <t>Kuning 44.25% - 88.51%</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Merah &lt; 43.42%</t>
+          <t>Merah &lt; 44.25%</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       <c r="P8" s="10" t="n">
         <v>1314</v>
       </c>
-      <c r="Q8" s="12">
+      <c r="Q8" s="13">
         <f>P8/B8</f>
         <v/>
       </c>
@@ -1846,7 +1846,7 @@
         <f>SUM(P7:P21)</f>
         <v/>
       </c>
-      <c r="Q22" s="12">
+      <c r="Q22" s="13">
         <f>P22/B22</f>
         <v/>
       </c>
@@ -1924,12 +1924,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-52):</t>
+          <t>Target Hari Ini (H-53):</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>86.84%</t>
+          <t>88.51%</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
       <c r="L66" s="10" t="n">
         <v>479</v>
       </c>
-      <c r="M66" s="12" t="n">
+      <c r="M66" s="13" t="n">
         <v>0.8805147058823529</v>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       <c r="L67" s="10" t="n">
         <v>445</v>
       </c>
-      <c r="M67" s="12" t="n">
+      <c r="M67" s="13" t="n">
         <v>0.8777120315581854</v>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       <c r="L68" s="10" t="n">
         <v>414</v>
       </c>
-      <c r="M68" s="12" t="n">
+      <c r="M68" s="13" t="n">
         <v>0.8752642706131079</v>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       <c r="L69" s="10" t="n">
         <v>424</v>
       </c>
-      <c r="M69" s="12" t="n">
+      <c r="M69" s="13" t="n">
         <v>0.8724279835390947</v>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
       <c r="L70" s="10" t="n">
         <v>347</v>
       </c>
-      <c r="M70" s="12" t="n">
+      <c r="M70" s="13" t="n">
         <v>0.871859296482412</v>
       </c>
     </row>
@@ -5052,7 +5052,7 @@
       <c r="L71" s="10" t="n">
         <v>349</v>
       </c>
-      <c r="M71" s="12" t="n">
+      <c r="M71" s="13" t="n">
         <v>0.8703241895261846</v>
       </c>
     </row>
@@ -5099,7 +5099,7 @@
       <c r="L72" s="10" t="n">
         <v>418</v>
       </c>
-      <c r="M72" s="12" t="n">
+      <c r="M72" s="13" t="n">
         <v>0.8690228690228691</v>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       <c r="L73" s="10" t="n">
         <v>423</v>
       </c>
-      <c r="M73" s="12" t="n">
+      <c r="M73" s="13" t="n">
         <v>0.8685831622176592</v>
       </c>
     </row>
@@ -8173,12 +8173,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-52):</t>
+          <t>Target Hari Ini (H-53):</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>86.84%</t>
+          <t>88.51%</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       <c r="L12" s="10" t="n">
         <v>2664</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="M12" s="13" t="n">
         <v>0.8783382789317506</v>
       </c>
     </row>
@@ -8575,7 +8575,7 @@
       <c r="L13" s="10" t="n">
         <v>2316</v>
       </c>
-      <c r="M13" s="12" t="n">
+      <c r="M13" s="13" t="n">
         <v>0.8687171792948237</v>
       </c>
     </row>
@@ -9384,12 +9384,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Target Hari Ini (H-52):</t>
+          <t>Target Hari Ini (H-53):</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>86.84%</t>
+          <t>88.51%</t>
         </is>
       </c>
     </row>
@@ -9533,7 +9533,7 @@
           <t>Tatoareng</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>0.8690476190476191</v>
       </c>
       <c r="D13" s="21" t="inlineStr">

</xml_diff>